<commit_message>
Activer la photo de couverture (branding.photoCouverture)
photo_couverture.png poussée sur main (3.8 Mo, 2000×1125) redimensionnée
et réencodée en JPEG qualité 85 (1400×787, 213 Ko) — largement suffisant
pour l'affichage ~240pt de la couverture, sans alourdir inutilement le PDF
régénéré côté navigateur à chaque génération. Original PNG conservé tel
quel à la racine, seule la version optimisée est servie depuis
content-pack/logos/.

RePSS_Entreprise_Reference.xlsx > Identite_Entreprise > photoCouverture
renseigné à "photo_couverture.jpg", entreprise.json recompilé (diff d'un
seul champ, vérifié). La couverture affiche maintenant la photo sous
l'encadré "Nom du chantier", vérifié visuellement.
</commit_message>
<xml_diff>
--- a/RePSS_Entreprise_Reference.xlsx
+++ b/RePSS_Entreprise_Reference.xlsx
@@ -722,7 +722,11 @@
           <t>photoCouverture</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>photo_couverture.jpg</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>photo/illustration page de couverture, sous l'encadré nom du chantier (optionnel)</t>

</xml_diff>